<commit_message>
forgot to save spreadsheets
</commit_message>
<xml_diff>
--- a/docs/RadioPacketTypes.xlsx
+++ b/docs/RadioPacketTypes.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="78">
   <si>
     <t xml:space="preserve">Packet Types</t>
   </si>
@@ -251,6 +251,9 @@
   </si>
   <si>
     <t xml:space="preserve">Debug</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h</t>
   </si>
 </sst>
 </file>
@@ -1077,6 +1080,9 @@
       <c r="C53" s="0" t="s">
         <v>76</v>
       </c>
+      <c r="D53" s="0" t="s">
+        <v>77</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="27">

</xml_diff>